<commit_message>
Update code with flowchart and shopify batch script
</commit_message>
<xml_diff>
--- a/Tracking_Results.xlsx
+++ b/Tracking_Results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,12 +473,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ILSC4001419607</t>
+          <t>52799210007416</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -488,119 +488,99 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>In Transit | Received at Motherhub_SAI_4 | THANE</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>29/04 00:00</t>
-        </is>
-      </c>
+          <t>Not Picked | Shipment not received from client | Lucknow_IndraNagar_D (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>22/04 16:39</t>
+          <t>20/04 12:26</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/ILSC4001419607</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210007416</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1323160104738</t>
+          <t>52799210008002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Delivered</t>
+          <t>Intransit</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Undelivered | Customer wants future delivery | MAA/RPM/LM1, Chennai, TAMIL NADU</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>07/05 00:00</t>
-        </is>
-      </c>
+          <t>Not Picked | Shipment not received from client | Lucknow_IndraNagar_D (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>02/05 13:48</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>09/05 13:46</t>
-        </is>
-      </c>
+          <t>21/04 11:03</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/1323160104738</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210008002</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>I79257402</t>
+          <t>52799210008271</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Delivered</t>
+          <t>Intransit</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Delivered | Delivered</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>07/05 00:00</t>
-        </is>
-      </c>
+          <t>Not Picked | Shipment not received from client | Lucknow_IndraNagar_D (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>02/05 13:52</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>08/05 14:24</t>
-        </is>
-      </c>
+          <t>21/04 14:06</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/I79257402</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210008271</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>21025858251910</t>
+          <t>52799210009542</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -610,77 +590,65 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>In Transit | Bag Received at Facility | Ayoor_Alayamon_D (Kerala)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>10/05 00:00</t>
-        </is>
-      </c>
+          <t>In Transit | Service Disruption | Imphal_Takyel_I (Manipur)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>02/05 12:17</t>
+          <t>23/04 14:11</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858251910</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210009542</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>21025858251932</t>
+          <t>52799210009483</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Delivered</t>
+          <t>Intransit</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Delivered | Delivered to consignee | Goa_PrabhuNagar_D (Goa)</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>12/05 00:00</t>
-        </is>
-      </c>
+          <t>Not Picked | Shipment not received from client | Lucknow_IndraNagar_D (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>02/05 12:17</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>08/05 14:01</t>
-        </is>
-      </c>
+          <t>23/04 10:55</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858251932</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210009483</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>21025858251921</t>
+          <t>52799210009391</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -690,35 +658,31 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>In Transit | Vehicle Departed | Pune_Sudhwadi_GW (Maharashtra)</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>10/05 00:00</t>
-        </is>
-      </c>
+          <t>In Transit | Shipment Received at Facility | Lucknow_Bhokapur_GW (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>02/05 12:17</t>
+          <t>23/04 14:06</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858251921</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210009391</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>21025857988570</t>
+          <t>52799210012316</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -728,35 +692,31 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Out For Delivery | Out for delivery | CumbumAP_RahamaniaNagar_D (Andhra Pradesh)</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>09/05 00:00</t>
-        </is>
-      </c>
+          <t>Pending | Shipment Received at Facility | Lucknow_IndraNagar_D (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>27/04 11:25</t>
+          <t>27/04 14:28</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025857988570</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210012316</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>21025858251943</t>
+          <t>52799210010625</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -766,77 +726,65 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>In Transit | Bag Received at Facility | Hyderabad_Medchal_GW (Telangana)</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>10/05 00:00</t>
-        </is>
-      </c>
+          <t>In Transit | Vehicle Departed | Guwahati_KaliPahar_GW (Assam)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>02/05 12:17</t>
+          <t>25/04 13:55</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858251943</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210010625</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>21025858251976</t>
+          <t>52799210012224</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Delivered</t>
+          <t>Intransit</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Undelivered | Consignee Unavailable | Tumsar_Dewhadi_DPP (Maharashtra)</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>09/05 00:00</t>
-        </is>
-      </c>
+          <t>In Transit | Vehicle Departed | Kannur_Payyanur_D (Kerala)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02/05 12:17</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>09/05 12:38</t>
-        </is>
-      </c>
+          <t>27/04 14:26</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858251976</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210012224</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>21025858048361</t>
+          <t>52799210012272</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -846,35 +794,31 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Out For Delivery | Out for delivery | Chennai_Nerkundram_D (Tamil Nadu)</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>09/05 00:00</t>
-        </is>
-      </c>
+          <t>Pending | Shipment Received at Facility | Lucknow_IndraNagar_D (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>28/04 10:20</t>
+          <t>27/04 14:24</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858048361</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210012272</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>21025858252002</t>
+          <t>52799210012132</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -884,35 +828,31 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>In Transit | Added to Bag | Vijayawada_Gudavalli_H (Andhra Pradesh)</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>11/05 00:00</t>
-        </is>
-      </c>
+          <t>In Transit | Added to Bag | Gurgaon_Tauru_GW (Haryana)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>02/05 12:17</t>
+          <t>27/04 14:28</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858252002</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210012132</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1323160103111</t>
+          <t>52799210012202</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -922,35 +862,31 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Out For Delivery | Out for Delivery | Chimakurthy, CHIMAKURTHY, ANDHRA PRADESH</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>05/05 00:00</t>
-        </is>
-      </c>
+          <t>In Transit | Vehicle Departed | Pune_BhamboliMIDC_H (Maharashtra)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>29/04 09:43</t>
+          <t>27/04 14:25</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/1323160103111</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210012202</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>21025858251965</t>
+          <t>52799210012176</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -960,35 +896,35 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>In Transit | Bag Received at Facility | Hyderabad_Medchal_GW (Telangana)</t>
+          <t>In Transit | Vehicle delayed - Controllable | Kanpur_Kataraghan_H (Uttar Pradesh)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>10/05 00:00</t>
+          <t>13/05 00:00</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>02/05 12:17</t>
+          <t>27/04 14:24</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858251965</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210012176</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>21025858252013</t>
+          <t>52799210012180</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -998,35 +934,35 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>In Transit | Added to Bag | Vijayawada_Gudavalli_H (Andhra Pradesh)</t>
+          <t>In Transit | Shipment Received at Facility | Lucknow_Bhokapur_GW (Uttar Pradesh)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11/05 00:00</t>
+          <t>18/05 00:00</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>02/05 12:17</t>
+          <t>27/04 14:24</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858252013</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210012180</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>21025858251991</t>
+          <t>52799210012283</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1036,73 +972,65 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Out For Delivery | Out for delivery | Phillaur_Parkashnagar_D (Punjab)</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>08/05 00:00</t>
-        </is>
-      </c>
+          <t>In Transit | Vehicle Departed | Nagpur_Khapari_GW (Maharashtra)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>02/05 12:17</t>
+          <t>27/04 14:28</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858251991</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210012283</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1323160104258</t>
+          <t>52799210014442</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>RTO</t>
+          <t>Intransit</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>RTO In Transit | RTO In Transit</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>04/05 00:00</t>
-        </is>
-      </c>
+          <t>In Transit | Vehicle delayed - Controllable | Bangalore_Hoskote_GW (Karnataka)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>01/05 12:26</t>
+          <t>30/04 13:31</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/1323160104258</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210014442</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>21025858251954</t>
+          <t>52799210014512</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1112,35 +1040,31 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Out For Delivery | Out for delivery | Lalpet_Kattumannarkoil1_D (Tamil Nadu)</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>09/05 00:00</t>
-        </is>
-      </c>
+          <t>In Transit | Added to Bag | Lucknow_Bhokapur_GW (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>02/05 12:17</t>
+          <t>30/04 13:30</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858251954</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210014512</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SF3337319830ITL</t>
+          <t>52799210014604</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1150,35 +1074,35 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Reached At Destination | Shipment is shipped to Shadowfax Warehouse | Visakhapatnam DC</t>
+          <t>Pending | Maximum attempts reached | Tiruvanamalai_VelNagar_D (Tamil Nadu)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>11/05 00:00</t>
+          <t>15/05 00:00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>02/05 19:18</t>
+          <t>01/05 14:30</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/SF3337319830ITL</t>
+          <t>https://www.delhivery.com/track-v2/package/52799210014604</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>21025858252035</t>
+          <t>52799210014615</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>iThink Logistics</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1188,25 +1112,439 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Out For Delivery | Out for delivery | Chilakaluripet_ChrlesChrch_DPP (Andhra Pradesh)</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>11/05 00:00</t>
-        </is>
-      </c>
+          <t>In Transit | Bag Received at Facility | Jhajjar_Policeline_I (Haryana)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>02/05 12:17</t>
+          <t>01/05 14:29</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://ithinklogistics.com/track/21025858252035</t>
-        </is>
-      </c>
+          <t>https://www.delhivery.com/track-v2/package/52799210014615</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>52799210014711</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Delhivery</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Intransit</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>In Transit | Vehicle delayed - Controllable | Pune_BhamboliMIDC_H (Maharashtra)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>01/05 14:29</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.delhivery.com/track-v2/package/52799210014711</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>52799210014722</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Delhivery</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Intransit</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>In Transit | Trip Arrived | Nagpur_Khapari_GW (Maharashtra)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>01/05 14:30</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.delhivery.com/track-v2/package/52799210014722</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>50207910018336</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>52799210014700</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Delhivery</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Intransit</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>In Transit | Shipment Received at Facility | Jaipur_Jaisinghpura_GW (Rajasthan)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>01/05 14:30</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.delhivery.com/track-v2/package/52799210014700</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>52799210014663</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Delhivery</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Intransit</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>In Transit | Bag Received at Facility | Tiruvalla_Ward6_D (Kerala)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>12/05 23:59</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>01/05 14:30</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://www.delhivery.com/track-v2/package/52799210014663</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>52799210007313</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Delhivery</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Intransit</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>In Transit | Vehicle Departed | Nagpur_Khapari_GW (Maharashtra)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>20/04 19:33</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://www.delhivery.com/track-v2/package/52799210007313</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>52799210006893</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Delhivery</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Intransit</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Dispatched | Out for delivery | Hyderabad_Ramnaspura_D (Telangana)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>16/05 00:00</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>20/04 19:31</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://www.delhivery.com/track-v2/package/52799210006893</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>52799210007162</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Delhivery</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Intransit</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>In Transit | Vehicle Departed | Ahmednagar_Nagapur_H (Maharashtra)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>20/04 19:29</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.delhivery.com/track-v2/package/52799210007162</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>52799210004454</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Delhivery</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Intransit</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>In Transit | Bag Received at Facility | Lucknow_Bhokapur_GW (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>16/04 13:40</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://www.delhivery.com/track-v2/package/52799210004454</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>52799210007254</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Delhivery</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Intransit</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Not Picked | Shipment not received from client | Lucknow_IndraNagar_D (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>20/04 12:23</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://www.delhivery.com/track-v2/package/52799210007254</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>52799210008024</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Delhivery</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Intransit</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Not Picked | Shipment not received from client | Lucknow_IndraNagar_D (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>21/04 11:03</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.delhivery.com/track-v2/package/52799210008024</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>52799210008945</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Delhivery</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Intransit</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>In Transit | Bag Added To Trip | Bhiwandi_Lonad_GW (Maharashtra)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>22/04 14:00</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://www.delhivery.com/track-v2/package/52799210008945</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1.32E+12</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>